<commit_message>
Legacy bug plans: v0.9.0 plans written out, L131 effect, new bug L230
- tools/gen_G.py rewrites 33 v0.9.0 plans cell by cell from the 465 file
  (118 entries); only L224, a change of method, stays described.
- L230 registered with its plan: the electricity current carbon tax and
  ETS outputs (results 16236-16251) never see the existing carbon price.
- Register text: L131 value effect (results 17161/17163), L129/L132/L133
  locations. Shared 465 reader in tools/xlsb465.py.
- Regenerated in place: BUGS.md, tracker, bugs document, register JSON,
  Documentation, Methods; counts 227 -> 228 patched in the deck, website
  page and QuickStart.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VSHkeKLNKwtFiko3pymStx
</commit_message>
<xml_diff>
--- a/excel_ai/Tracking_Legacy_Bugs_v1.0.0.xlsx
+++ b/excel_ai/Tracking_Legacy_Bugs_v1.0.0.xlsx
@@ -13,9 +13,9 @@
     <workbookView activeTab="0" xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{39055DA2-BF7E-4A30-86A0-0114139A7EB4}"/>
   </bookViews>
   <sheets>
-    <sheet name="ReadMe" sheetId="32" r:id="rId14"/>
-    <sheet name="Bugs" sheetId="33" r:id="rId15"/>
-    <sheet name="Issues" sheetId="34" r:id="rId16"/>
+    <sheet name="ReadMe" sheetId="38" r:id="rId14"/>
+    <sheet name="Bugs" sheetId="39" r:id="rId15"/>
+    <sheet name="Issues" sheetId="40" r:id="rId16"/>
     <sheet name="CPAT_issues" sheetId="1" r:id="rId1"/>
     <sheet name="CPAT-MT" sheetId="3" r:id="rId2"/>
     <sheet name="Mit+Disn_DeepDive" sheetId="6" r:id="rId3"/>
@@ -4462,7 +4462,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">L (227)</t>
+          <t xml:space="preserve">L (228)</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -4565,7 +4565,7 @@
   <sheetPr>
     <tabColor rgb="FF1F4E78"/>
   </sheetPr>
-  <dimension ref="A1:V270"/>
+  <dimension ref="A1:V271"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="8.9" customWidth="1"/>
@@ -17599,7 +17599,7 @@
       <c r="H128" s="0"/>
       <c r="I128" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in legacy 465 (not marked fixed by the CPAT team). Where: Mitigation rows 2785-2788, 2947-2951, 7883-7886 (against 2743, 2745).</t>
+          <t xml:space="preserve">Open in legacy 465 (not marked fixed by the CPAT team). Where: Mitigation rows 2785-2788, 2947-2951 (policy 9101-9104, 9263-9267), against 2743, 2745.</t>
         </is>
       </c>
       <c r="J128" s="4" t="inlineStr">
@@ -17635,7 +17635,7 @@
       </c>
       <c r="Q128" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mitigation rows 2785-2788, 2947-2951, 7883-7886 (against 2743, 2745)</t>
+          <t xml:space="preserve">Mitigation rows 2785-2788, 2947-2951 (policy 9101-9104, 9263-9267), against 2743, 2745</t>
         </is>
       </c>
       <c r="R128" s="3" t="inlineStr">
@@ -17645,7 +17645,7 @@
       </c>
       <c r="S128" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">In rows 2785-2788, 2947-2951 and 7883-7886 drop the + L2743 term (L2745 already includes it); policy rows the same (+6,316).</t>
+          <t xml:space="preserve">In rows 2785-2788 and 2947-2951 drop the + L2743 term (L2745 already includes it); policy rows the same (+6,316: 9101-9104, 9263-9267).</t>
         </is>
       </c>
       <c r="T128" s="3" t="inlineStr">
@@ -17799,7 +17799,7 @@
       <c r="H130" s="0"/>
       <c r="I130" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in legacy 465 (not marked fixed by the CPAT team). Where: Mitigation rows 466, 2442, 16170 (gdp.pre.lvl); 7722, 7742, 7985 (sub.new.usd); 7638-13962 (rev.ctr.coa).</t>
+          <t xml:space="preserve">Open in legacy 465 (not marked fixed by the CPAT team). Where: Mitigation H466, H2442 (gdp.pre.lvl); H7736:H7737, H7756:H7757, H7999:H8000 and policy copies (sub.new.usd/pct; read by results rows 17161, 17163); H7652:H7660, H13968:H13976 (rev.ctr.coa).</t>
         </is>
       </c>
       <c r="J130" s="4" t="inlineStr">
@@ -17835,22 +17835,22 @@
       </c>
       <c r="Q130" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mitigation rows 466, 2442, 16170 (gdp.pre.lvl); 7722, 7742, 7985 (sub.new.usd); 7638-13962 (rev.ctr.coa)</t>
+          <t xml:space="preserve">Mitigation H466, H2442 (gdp.pre.lvl); H7736:H7737, H7756:H7757, H7999:H8000 and policy copies (sub.new.usd/pct; read by results rows 17161, 17163); H7652:H7660, H13968:H13976 (rev.ctr.coa)</t>
         </is>
       </c>
       <c r="R130" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Legacy reuses a code for other quantities: gdp.pre.lvl for ln(GDP pc), GDP in $mn and in bn US$; sub.new.usd for revenue subtotals; rev.ctr.coa for the gasoline to electricity rows. A lookup by code finds the first row only. Found by the codes crosswalk (v0.7.1).</t>
+          <t xml:space="preserve">Legacy reuses a code for other quantities: gdp.pre.lvl for ln(GDP pc), GDP in $mn and in bn US$; sub.new.usd for revenue subtotals; rev.ctr.coa for the gasoline to electricity rows. A lookup by code finds the first row only. Value effect: results rows 17161/17163 (revenues, % of GDP) look up sub.new.pct and find the carbon-price subtotal (rows 7737/14053) instead of the total revenue (8013/14329) that their US$ partners 17160/17162 read; Egypt, carbon tax, 2040: 0.0015% of GDP where the total is -0.0215% (found by the cell plan, 2026-10-29). Found by the codes crosswalk (v0.7.1).</t>
         </is>
       </c>
       <c r="S130" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Give each row its own code (e.g. gdp.pre.ln, gdp.pre.mn; sub.new.usd only on its own subtotal).</t>
+          <t xml:space="preserve">Give each row its own code (ln.gdppc on row 466; rev.ctx.tot, rev.exc.tot, rev.tot.tot on the three revenue subtotals; the fuel token on the rev.ctr rows), and let results rows 17161/17163 read rev.new.pct (the total).</t>
         </is>
       </c>
       <c r="T130" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lookups by code (MTOutputs, the data link) return the first row of a reused code.</t>
+          <t xml:space="preserve">Results rows 17161, 17163 and 17165 (revenues in % of GDP) report the carbon-price subtotal instead of the total revenue; lookups by code (MTOutputs, the data link) return the first row of a reused code.</t>
         </is>
       </c>
       <c r="U130" s="3"/>
@@ -17899,7 +17899,7 @@
       <c r="H131" s="0"/>
       <c r="I131" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in legacy 465 (not marked fixed by the CPAT team). Where: Mitigation rows 7606, 13922 (oc.tot.); em.pm2.All.&lt;sector&gt; rows.</t>
+          <t xml:space="preserve">Open in legacy 465 (not marked fixed by the CPAT team). Where: Mitigation H6668:H7397 (the All rows of the 8 pollutant blocks) and policy H12984:H13713; 67 codes with an empty token (H2320, H3225:H3233, H3315:H3323, H3474:H3482, H3643:H3644, H7589:H7590, H7620, G17215 and policy copies).</t>
         </is>
       </c>
       <c r="J131" s="4" t="inlineStr">
@@ -17935,7 +17935,7 @@
       </c>
       <c r="Q131" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mitigation rows 7606, 13922 (oc.tot.); em.pm2.All.&lt;sector&gt; rows</t>
+          <t xml:space="preserve">Mitigation H6668:H7397 (the All rows of the 8 pollutant blocks) and policy H12984:H13713; 67 codes with an empty token (H2320, H3225:H3233, H3315:H3323, H3474:H3482, H3643:H3644, H7589:H7590, H7620, G17215 and policy copies)</t>
         </is>
       </c>
       <c r="R131" s="3" t="inlineStr">
@@ -17953,7 +17953,11 @@
           <t xml:space="preserve">Lookups of the protocol codes fail.</t>
         </is>
       </c>
-      <c r="U131" s="3"/>
+      <c r="U131" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L230</t>
+        </is>
+      </c>
       <c r="V131" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Legacy CPAT bugs document</t>
@@ -17999,7 +18003,7 @@
       <c r="H132" s="0"/>
       <c r="I132" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in legacy 465 (not marked fixed by the CPAT team). Where: Mitigation rows 7606, 13922 and the GHG total rows (nox.tot).</t>
+          <t xml:space="preserve">Open in legacy 465 (not marked fixed by the CPAT team). Where: Mitigation H7614, H7620 (policy H13930, H13936); readers G18242, G18247 (MTOutputs E84, E89).</t>
         </is>
       </c>
       <c r="J132" s="4" t="inlineStr">
@@ -18035,7 +18039,7 @@
       </c>
       <c r="Q132" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mitigation rows 7606, 13922 and the GHG total rows (nox.tot)</t>
+          <t xml:space="preserve">Mitigation H7614, H7620 (policy H13930, H13936); readers G18242, G18247 (MTOutputs E84, E89)</t>
         </is>
       </c>
       <c r="R132" s="3" t="inlineStr">
@@ -27319,20 +27323,32 @@
     <row r="229">
       <c r="A229" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">L230</t>
         </is>
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Version-log rows rewritten with the current version</t>
-        </is>
-      </c>
-      <c r="C229" s="4"/>
-      <c r="D229" s="4"/>
-      <c r="E229" s="4"/>
-      <c r="F229" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Solved</t>
+          <t xml:space="preserve">Electricity: current carbon tax and ETS outputs never see the existing carbon price</t>
+        </is>
+      </c>
+      <c r="C229" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">465</t>
+        </is>
+      </c>
+      <c r="D229" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-29</t>
+        </is>
+      </c>
+      <c r="E229" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 (Low)</t>
+        </is>
+      </c>
+      <c r="F229" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
         </is>
       </c>
       <c r="G229" s="0" t="inlineStr">
@@ -27340,15 +27356,15 @@
           <t xml:space="preserve">Stephen (CPAT-AI)</t>
         </is>
       </c>
-      <c r="H229" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CPAT-AI (prototype)</t>
-        </is>
-      </c>
-      <c r="I229" s="3"/>
+      <c r="H229" s="0"/>
+      <c r="I229" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open in legacy 465 (not marked fixed by the CPAT team). Where: Mitigation L16236:AE16237 (current carbon tax, electricity), L16250:AE16251 (current ETS, electricity); published by MTOutputs K229:K230, K242:K243 and rows 16702-16703.</t>
+        </is>
+      </c>
       <c r="J229" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prototype bug</t>
+          <t xml:space="preserve">Legacy bug</t>
         </is>
       </c>
       <c r="K229" s="4"/>
@@ -27364,43 +27380,59 @@
       </c>
       <c r="N229" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fixed (v0.0.3-v0.0.4 / v0.0.5)</t>
+          <t xml:space="preserve">Not built in the prototype (it has no current-carbon-price output for electricity): nothing replicated.</t>
         </is>
       </c>
       <c r="O229" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Closed</t>
-        </is>
-      </c>
-      <c r="P229" s="4"/>
-      <c r="Q229" s="3"/>
+          <t xml:space="preserve">Open in legacy</t>
+        </is>
+      </c>
+      <c r="P229" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="Q229" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mitigation L16236:AE16237 (current carbon tax, electricity), L16250:AE16251 (current ETS, electricity); published by MTOutputs K229:K230, K242:K243 and rows 16702-16703</t>
+        </is>
+      </c>
       <c r="R229" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The builders wrote earlier version-log rows with the current version number.</t>
+          <t xml:space="preserve">The results rows for the current (existing) carbon tax and ETS on electricity look up a power-price row by code. Rows 16236/16237 (current carbon tax) find ctx.ind.ecy.t / ctx.res.ecy.t, the rows "Policy (usually carbon price)" 3643/3614, which carry the new policy's carbon cost (row 3395, from the "total new policy" rows 2468, 2537, 2698): 0 in scenario 1 by construction. Rows 16250/16251 (current ETS) look up ets.ind.ecy.t.1 / ets.res.ecy.t.1, which no row carries (IFNA 0). The existing carbon tax and ETS of the power fuels (rows 2462-2463 coal, 2531-2532 gas, 2692-2693 oil) never reach these outputs, so a country with a carbon tax or ETS on power reports 0 for electricity.</t>
         </is>
       </c>
       <c r="S229" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Each row has its own version; old workbooks left as shipped.</t>
-        </is>
-      </c>
-      <c r="T229" s="3"/>
-      <c r="U229" s="3"/>
+          <t xml:space="preserve">Rows 3385-3395: the new policy's carbon cost per kWh consumed (fuel cost per GJ / efficiency x generation share, / transmission factor J3395); the same chain on the existing carbon price rows.</t>
+        </is>
+      </c>
+      <c r="T229" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None for Egypt (no existing carbon tax or ETS on power). Elsewhere the current carbon tax and ETS on electricity (results 16236-16251, MTOutputs K229:K230 and K242:K243, rows 16702-16703) show the existing carbon price per kWh instead of 0. Industry and residential get the same value: the price is upstream, before pass-through and VAT.</t>
+        </is>
+      </c>
+      <c r="U229" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L132</t>
+        </is>
+      </c>
       <c r="V229" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Documentation, appendix</t>
+          <t xml:space="preserve">Legacy CPAT bugs document</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2</t>
+          <t xml:space="preserve">M1</t>
         </is>
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Power: VAT left out on the policy term</t>
+          <t xml:space="preserve">Version-log rows rewritten with the current version</t>
         </is>
       </c>
       <c r="C230" s="4"/>
@@ -27440,7 +27472,7 @@
       </c>
       <c r="N230" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fixed (v0.1.05 / v0.1.06)</t>
+          <t xml:space="preserve">Fixed (v0.0.3-v0.0.4 / v0.0.5)</t>
         </is>
       </c>
       <c r="O230" s="4" t="inlineStr">
@@ -27452,12 +27484,12 @@
       <c r="Q230" s="3"/>
       <c r="R230" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The end-user price added the policy cost without VAT; legacy row 3614 charges VAT.</t>
+          <t xml:space="preserve">The builders wrote earlier version-log rows with the current version number.</t>
         </is>
       </c>
       <c r="S230" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">VAT on the policy term as legacy (no effect for Egypt, VAT 0).</t>
+          <t xml:space="preserve">Each row has its own version; old workbooks left as shipped.</t>
         </is>
       </c>
       <c r="T230" s="3"/>
@@ -27471,12 +27503,12 @@
     <row r="231">
       <c r="A231" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M3</t>
+          <t xml:space="preserve">M2</t>
         </is>
       </c>
       <c r="B231" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Power: long-term storage allocation left out</t>
+          <t xml:space="preserve">Power: VAT left out on the policy term</t>
         </is>
       </c>
       <c r="C231" s="4"/>
@@ -27528,12 +27560,12 @@
       <c r="Q231" s="3"/>
       <c r="R231" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The legacy note "incomplete" was read as "not applied".</t>
+          <t xml:space="preserve">The end-user price added the policy cost without VAT; legacy row 3614 charges VAT.</t>
         </is>
       </c>
       <c r="S231" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The 33% allocation is applied once.</t>
+          <t xml:space="preserve">VAT on the policy term as legacy (no effect for Egypt, VAT 0).</t>
         </is>
       </c>
       <c r="T231" s="3"/>
@@ -27547,12 +27579,12 @@
     <row r="232">
       <c r="A232" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M4</t>
+          <t xml:space="preserve">M3</t>
         </is>
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Power: VRE share without other renewables</t>
+          <t xml:space="preserve">Power: long-term storage allocation left out</t>
         </is>
       </c>
       <c r="C232" s="4"/>
@@ -27604,12 +27636,12 @@
       <c r="Q232" s="3"/>
       <c r="R232" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Legacy row 3851 also counts other renewables.</t>
+          <t xml:space="preserve">The legacy note "incomplete" was read as "not applied".</t>
         </is>
       </c>
       <c r="S232" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Follows legacy (other renewables 0 for Egypt).</t>
+          <t xml:space="preserve">The 33% allocation is applied once.</t>
         </is>
       </c>
       <c r="T232" s="3"/>
@@ -27623,12 +27655,12 @@
     <row r="233">
       <c r="A233" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M5</t>
+          <t xml:space="preserve">M4</t>
         </is>
       </c>
       <c r="B233" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Defined name clashed with a LAMBDA name</t>
+          <t xml:space="preserve">Power: VRE share without other renewables</t>
         </is>
       </c>
       <c r="C233" s="4"/>
@@ -27668,7 +27700,7 @@
       </c>
       <c r="N233" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fixed (v0.1.07 build / v0.1.07)</t>
+          <t xml:space="preserve">Fixed (v0.1.05 / v0.1.06)</t>
         </is>
       </c>
       <c r="O233" s="4" t="inlineStr">
@@ -27680,12 +27712,12 @@
       <c r="Q233" s="3"/>
       <c r="R233" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The defined name ETSSemi equals the LAMBDA ETSSEMI ignoring case and gave #NAME?; the ETS goal seek stopped converging.</t>
+          <t xml:space="preserve">Legacy row 3851 also counts other renewables.</t>
         </is>
       </c>
       <c r="S233" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Renamed SemiEl; the builder asserts that no defined name equals a LAMBDA name.</t>
+          <t xml:space="preserve">Follows legacy (other renewables 0 for Egypt).</t>
         </is>
       </c>
       <c r="T233" s="3"/>
@@ -27699,12 +27731,12 @@
     <row r="234">
       <c r="A234" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M6</t>
+          <t xml:space="preserve">M5</t>
         </is>
       </c>
       <c r="B234" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Power ETS revenue valued at the tax-equivalent price</t>
+          <t xml:space="preserve">Defined name clashed with a LAMBDA name</t>
         </is>
       </c>
       <c r="C234" s="4"/>
@@ -27744,7 +27776,7 @@
       </c>
       <c r="N234" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fixed (v0.1.05 / v0.1.09)</t>
+          <t xml:space="preserve">Fixed (v0.1.07 build / v0.1.07)</t>
         </is>
       </c>
       <c r="O234" s="4" t="inlineStr">
@@ -27756,12 +27788,12 @@
       <c r="Q234" s="3"/>
       <c r="R234" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Power new-policy revenue (ccpav x consumption) valued the ETS at the tax-equivalent price, about 10% high at Medium volatility.</t>
+          <t xml:space="preserve">The defined name ETSSemi equals the LAMBDA ETSSEMI ignoring case and gave #NAME?; the ETS goal seek stopped converging.</t>
         </is>
       </c>
       <c r="S234" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Revenue by generation type (prnew) with the ETS at the permit price; rcarb kept as a memo.</t>
+          <t xml:space="preserve">Renamed SemiEl; the builder asserts that no defined name equals a LAMBDA name.</t>
         </is>
       </c>
       <c r="T234" s="3"/>
@@ -27775,12 +27807,12 @@
     <row r="235">
       <c r="A235" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M7</t>
+          <t xml:space="preserve">M6</t>
         </is>
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stale texts in the workbook and notes</t>
+          <t xml:space="preserve">Power ETS revenue valued at the tax-equivalent price</t>
         </is>
       </c>
       <c r="C235" s="4"/>
@@ -27820,7 +27852,7 @@
       </c>
       <c r="N235" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fixed (v0.1.08 / v0.1.09)</t>
+          <t xml:space="preserve">Fixed (v0.1.05 / v0.1.09)</t>
         </is>
       </c>
       <c r="O235" s="4" t="inlineStr">
@@ -27832,12 +27864,12 @@
       <c r="Q235" s="3"/>
       <c r="R235" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Section 12 and 13 notes said power was not included; PowerPaths said interim data; data sheets named old extractors; method notes described earlier versions.</t>
+          <t xml:space="preserve">Power new-policy revenue (ccpav x consumption) valued the ETS at the tax-equivalent price, about 10% high at Medium volatility.</t>
         </is>
       </c>
       <c r="S235" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Texts updated; the check now scans the workbook texts for stale statements and missing file references.</t>
+          <t xml:space="preserve">Revenue by generation type (prnew) with the ETS at the permit price; rcarb kept as a memo.</t>
         </is>
       </c>
       <c r="T235" s="3"/>
@@ -27851,12 +27883,12 @@
     <row r="236">
       <c r="A236" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M8</t>
+          <t xml:space="preserve">M7</t>
         </is>
       </c>
       <c r="B236" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">LegacyDiff rows out of date</t>
+          <t xml:space="preserve">Stale texts in the workbook and notes</t>
         </is>
       </c>
       <c r="C236" s="4"/>
@@ -27896,7 +27928,7 @@
       </c>
       <c r="N236" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fixed (v0.1.09 / v0.2.2)</t>
+          <t xml:space="preserve">Fixed (v0.1.08 / v0.1.09)</t>
         </is>
       </c>
       <c r="O236" s="4" t="inlineStr">
@@ -27908,12 +27940,12 @@
       <c r="Q236" s="3"/>
       <c r="R236" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing carbon pricing was still listed as "Not modelled"; the formula-structure row described the LAMBDA right column of v0.1.07.</t>
+          <t xml:space="preserve">Section 12 and 13 notes said power was not included; PowerPaths said interim data; data sheets named old extractors; method notes described earlier versions.</t>
         </is>
       </c>
       <c r="S236" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rows updated; the check scans for these phrases.</t>
+          <t xml:space="preserve">Texts updated; the check now scans the workbook texts for stale statements and missing file references.</t>
         </is>
       </c>
       <c r="T236" s="3"/>
@@ -27927,12 +27959,12 @@
     <row r="237">
       <c r="A237" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M9</t>
+          <t xml:space="preserve">M8</t>
         </is>
       </c>
       <c r="B237" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Legacy comparison note from v0.1.01</t>
+          <t xml:space="preserve">LegacyDiff rows out of date</t>
         </is>
       </c>
       <c r="C237" s="4"/>
@@ -27972,7 +28004,7 @@
       </c>
       <c r="N237" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fixed (v0.1.02-v0.1.09 / v0.2.2)</t>
+          <t xml:space="preserve">Fixed (v0.1.09 / v0.2.2)</t>
         </is>
       </c>
       <c r="O237" s="4" t="inlineStr">
@@ -27984,12 +28016,12 @@
       <c r="Q237" s="3"/>
       <c r="R237" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">legacy_comparison described the v0.1.01 baseline and its script wrote a different file name.</t>
+          <t xml:space="preserve">Existing carbon pricing was still listed as "Not modelled"; the formula-structure row described the LAMBDA right column of v0.1.07.</t>
         </is>
       </c>
       <c r="S237" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Re-run on v0.2.2 (legacy_comparison_v6_4.md).</t>
+          <t xml:space="preserve">Rows updated; the check scans for these phrases.</t>
         </is>
       </c>
       <c r="T237" s="3"/>
@@ -28003,12 +28035,12 @@
     <row r="238">
       <c r="A238" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M10</t>
+          <t xml:space="preserve">M9</t>
         </is>
       </c>
       <c r="B238" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Total rows labelled "All subsectors"</t>
+          <t xml:space="preserve">Legacy comparison note from v0.1.01</t>
         </is>
       </c>
       <c r="C238" s="4"/>
@@ -28048,7 +28080,7 @@
       </c>
       <c r="N238" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fixed (v0.1.09 / v0.2.3)</t>
+          <t xml:space="preserve">Fixed (v0.1.02-v0.1.09 / v0.2.2)</t>
         </is>
       </c>
       <c r="O238" s="4" t="inlineStr">
@@ -28060,12 +28092,12 @@
       <c r="Q238" s="3"/>
       <c r="R238" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Since v0.1.09 the totals (fuel use, CO2, revenues) include power, but the label of the sector code all still said "All subsectors".</t>
+          <t xml:space="preserve">legacy_comparison described the v0.1.01 baseline and its script wrote a different file name.</t>
         </is>
       </c>
       <c r="S238" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Label "All sectors".</t>
+          <t xml:space="preserve">Re-run on v0.2.2 (legacy_comparison_v6_4.md).</t>
         </is>
       </c>
       <c r="T238" s="3"/>
@@ -28079,12 +28111,12 @@
     <row r="239">
       <c r="A239" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M11</t>
+          <t xml:space="preserve">M10</t>
         </is>
       </c>
       <c r="B239" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Macros read 19 year columns</t>
+          <t xml:space="preserve">Total rows labelled "All subsectors"</t>
         </is>
       </c>
       <c r="C239" s="4"/>
@@ -28124,7 +28156,7 @@
       </c>
       <c r="N239" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fixed (v0.2.3 build / v0.2.3)</t>
+          <t xml:space="preserve">Fixed (v0.1.09 / v0.2.3)</t>
         </is>
       </c>
       <c r="O239" s="4" t="inlineStr">
@@ -28136,12 +28168,12 @@
       <c r="Q239" s="3"/>
       <c r="R239" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The VBA module had the number of years (NYEARS = 19, 2022-2040) as a constant; with the horizon to 2041 the batch run and CheckBatchRun would have stored and compared one year too few (found by the check).</t>
+          <t xml:space="preserve">Since v0.1.09 the totals (fuel use, CO2, revenues) include power, but the label of the sector code all still said "All subsectors".</t>
         </is>
       </c>
       <c r="S239" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">NYEARS = 20; the builder now asserts that it equals the number of model years.</t>
+          <t xml:space="preserve">Label "All sectors".</t>
         </is>
       </c>
       <c r="T239" s="3"/>
@@ -28155,12 +28187,12 @@
     <row r="240">
       <c r="A240" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M12</t>
+          <t xml:space="preserve">M11</t>
         </is>
       </c>
       <c r="B240" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sheet Lambdas: formula texts named merged sheets</t>
+          <t xml:space="preserve">Macros read 19 year columns</t>
         </is>
       </c>
       <c r="C240" s="4"/>
@@ -28200,7 +28232,7 @@
       </c>
       <c r="N240" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fixed (v0.3.6 / v0.3.13)</t>
+          <t xml:space="preserve">Fixed (v0.2.3 build / v0.2.3)</t>
         </is>
       </c>
       <c r="O240" s="4" t="inlineStr">
@@ -28212,12 +28244,12 @@
       <c r="Q240" s="3"/>
       <c r="R240" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The tab merge of v0.3.6 re-pointed every formula but not the formula texts of sheet Lambdas (column F), so the rows reading the power and price inputs named Inputs_power / Inputs_prices, which no longer exist; copied into Mitigation they gave #REF! (found by the full check, variant B).</t>
+          <t xml:space="preserve">The VBA module had the number of years (NYEARS = 19, 2022-2040) as a constant; with the horizon to 2041 the batch run and CheckBatchRun would have stored and compared one year too few (found by the check).</t>
         </is>
       </c>
       <c r="S240" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">merge_tabs re-points the texts too; the full check copies them over every row (variant B).</t>
+          <t xml:space="preserve">NYEARS = 20; the builder now asserts that it equals the number of model years.</t>
         </is>
       </c>
       <c r="T240" s="3"/>
@@ -28231,12 +28263,12 @@
     <row r="241">
       <c r="A241" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M13</t>
+          <t xml:space="preserve">M12</t>
         </is>
       </c>
       <c r="B241" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Road vehicle feebate counted the carbon price twice</t>
+          <t xml:space="preserve">Sheet Lambdas: formula texts named merged sheets</t>
         </is>
       </c>
       <c r="C241" s="4"/>
@@ -28276,7 +28308,7 @@
       </c>
       <c r="N241" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fixed (v0.3.5 / v0.4.16)</t>
+          <t xml:space="preserve">Fixed (v0.3.6 / v0.3.13)</t>
         </is>
       </c>
       <c r="O241" s="4" t="inlineStr">
@@ -28288,12 +28320,12 @@
       <c r="Q241" s="3"/>
       <c r="R241" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The vehicle feebate rate of the engineer road model added the carbon price x road feebate share in every policy scenario, although the carbon tax is in the fuel price already (legacy adds the shadow carbon price, 0 under explicit pricing).</t>
+          <t xml:space="preserve">The tab merge of v0.3.6 re-pointed every formula but not the formula texts of sheet Lambdas (column F), so the rows reading the power and price inputs named Inputs_power / Inputs_prices, which no longer exist; copied into Mitigation they gave #REF! (found by the full check, variant B).</t>
         </is>
       </c>
       <c r="S241" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The road regulation shadow price (reg.rod) replaces it; 0 under explicit pricing.</t>
+          <t xml:space="preserve">merge_tabs re-points the texts too; the full check copies them over every row (variant B).</t>
         </is>
       </c>
       <c r="T241" s="3"/>
@@ -28307,12 +28339,12 @@
     <row r="242">
       <c r="A242" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M14</t>
+          <t xml:space="preserve">M13</t>
         </is>
       </c>
       <c r="B242" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">LAMBDA library texts named a merged-away sheet</t>
+          <t xml:space="preserve">Road vehicle feebate counted the carbon price twice</t>
         </is>
       </c>
       <c r="C242" s="4"/>
@@ -28352,7 +28384,7 @@
       </c>
       <c r="N242" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fixed (v0.4.2 / v0.5.3)</t>
+          <t xml:space="preserve">Fixed (v0.3.5 / v0.4.16)</t>
         </is>
       </c>
       <c r="O242" s="4" t="inlineStr">
@@ -28364,12 +28396,12 @@
       <c r="Q242" s="3"/>
       <c r="R242" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The 21 LAMBDA-library texts of the power pollutant rows (sheet Lambdas, column C) still named the sheet Inputs_power: the v0.3.13 fix (M12) re-pointed the texts only on sheets that stay in place, and Lambdas is an appended block since v0.4.2; pasted, they gave #NAME?.</t>
+          <t xml:space="preserve">The vehicle feebate rate of the engineer road model added the carbon price x road feebate share in every policy scenario, although the carbon tax is in the fuel price already (legacy adds the shadow carbon price, 0 under explicit pricing).</t>
         </is>
       </c>
       <c r="S242" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">merge_tabs re-points the Lambdas texts of an appended block too (host Mitigation); the full check lists any text naming a merged-away sheet.</t>
+          <t xml:space="preserve">The road regulation shadow price (reg.rod) replaces it; 0 under explicit pricing.</t>
         </is>
       </c>
       <c r="T242" s="3"/>
@@ -28383,12 +28415,12 @@
     <row r="243">
       <c r="A243" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M15</t>
+          <t xml:space="preserve">M14</t>
         </is>
       </c>
       <c r="B243" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Section 18: VAT on efficient prices at the 2022 general rate in every year</t>
+          <t xml:space="preserve">LAMBDA library texts named a merged-away sheet</t>
         </is>
       </c>
       <c r="C243" s="4"/>
@@ -28428,7 +28460,7 @@
       </c>
       <c r="N243" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fixed (v0.9.1 (Coded CPAT) / v0.9.2)</t>
+          <t xml:space="preserve">Fixed (v0.4.2 / v0.5.3)</t>
         </is>
       </c>
       <c r="O243" s="4" t="inlineStr">
@@ -28440,20 +28472,16 @@
       <c r="Q243" s="3"/>
       <c r="R243" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The defined name VatGen was one fixed cell, the general VAT rate (VAT_WEO) of 2022; every year of the energy-subsidy (vatext) and efficient-price (vat.cost) rows applied it, whatever the year's rate.</t>
+          <t xml:space="preserve">The 21 LAMBDA-library texts of the power pollutant rows (sheet Lambdas, column C) still named the sheet Inputs_power: the v0.3.13 fix (M12) re-pointed the texts only on sheets that stay in place, and Lambdas is an appended block since v0.4.2; pasted, they gave #NAME?.</t>
         </is>
       </c>
       <c r="S243" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">New section-18 row vatgen: VAT_WEO of the year up to LastHistPriceYear, the last historical rate held after it (user assumption 2026-10-29); column D keeps the consumer flag x household share. Egypt unchanged (14% throughout). Legacy: the subsidy block uses the year's rate (L17787), so the vatext part was introduced in v0.9.0; the efficient-price part is legacy bug L225.</t>
+          <t xml:space="preserve">merge_tabs re-points the Lambdas texts of an appended block too (host Mitigation); the full check lists any text naming a merged-away sheet.</t>
         </is>
       </c>
       <c r="T243" s="3"/>
-      <c r="U243" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">L225, I120</t>
-        </is>
-      </c>
+      <c r="U243" s="3"/>
       <c r="V243" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Documentation, appendix</t>
@@ -28463,12 +28491,12 @@
     <row r="244">
       <c r="A244" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M16</t>
+          <t xml:space="preserve">M15</t>
         </is>
       </c>
       <c r="B244" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Road: freight BEV feebate valued at the ICEV truck's distance</t>
+          <t xml:space="preserve">Section 18: VAT on efficient prices at the 2022 general rate in every year</t>
         </is>
       </c>
       <c r="C244" s="4"/>
@@ -28520,18 +28548,18 @@
       <c r="Q244" s="3"/>
       <c r="R244" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">trfbvfb.fre.bev multiplied by the ICEV discounted km (trdkmfrei); the passenger and 2-3 wheeler BEV feebates use the BEV distance.</t>
+          <t xml:space="preserve">The defined name VatGen was one fixed cell, the general VAT rate (VAT_WEO) of 2022; every year of the energy-subsidy (vatext) and efficient-price (vat.cost) rows applied it, whatever the year's rate.</t>
         </is>
       </c>
       <c r="S244" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The freight BEV discounted km (trdkmfreb.fre.bev, legacy row 4630). Engineer road model only. In legacy too: L226.</t>
+          <t xml:space="preserve">New section-18 row vatgen: VAT_WEO of the year up to LastHistPriceYear, the last historical rate held after it (user assumption 2026-10-29); column D keeps the consumer flag x household share. Egypt unchanged (14% throughout). Legacy: the subsidy block uses the year's rate (L17787), so the vatext part was introduced in v0.9.0; the efficient-price part is legacy bug L225.</t>
         </is>
       </c>
       <c r="T244" s="3"/>
       <c r="U244" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">L226</t>
+          <t xml:space="preserve">L225, I120</t>
         </is>
       </c>
       <c r="V244" s="3" t="inlineStr">
@@ -28543,12 +28571,12 @@
     <row r="245">
       <c r="A245" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M17</t>
+          <t xml:space="preserve">M16</t>
         </is>
       </c>
       <c r="B245" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Road: plug-in hybrid cost mixed BEV capital cost with ICEV insurance and maintenance</t>
+          <t xml:space="preserve">Road: freight BEV feebate valued at the ICEV truck's distance</t>
         </is>
       </c>
       <c r="C245" s="4"/>
@@ -28600,18 +28628,18 @@
       <c r="Q245" s="3"/>
       <c r="R245" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">trtcfp.pas.phv took the BEV depreciation and salvage with the ICEV insurance and maintenance (insurance on the ICEV price).</t>
+          <t xml:space="preserve">trfbvfb.fre.bev multiplied by the ICEV discounted km (trdkmfrei); the passenger and 2-3 wheeler BEV feebates use the BEV distance.</t>
         </is>
       </c>
       <c r="S245" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">One price basis (user 2026-10-29; no PHEV price in the data): new row trimphv.pas.phv, insurance on the BEV price with the ICEV maintenance per km and the ICEV distance. Engineer road model only. In legacy too: L227 (with L41, the range anxiety).</t>
+          <t xml:space="preserve">The freight BEV discounted km (trdkmfreb.fre.bev, legacy row 4630). Engineer road model only. In legacy too: L226.</t>
         </is>
       </c>
       <c r="T245" s="3"/>
       <c r="U245" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">L227, L41</t>
+          <t xml:space="preserve">L226</t>
         </is>
       </c>
       <c r="V245" s="3" t="inlineStr">
@@ -28623,12 +28651,12 @@
     <row r="246">
       <c r="A246" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M18</t>
+          <t xml:space="preserve">M17</t>
         </is>
       </c>
       <c r="B246" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Road: bus electricity scaled by the bus energy of every fuel (withdrawn: not a bug)</t>
+          <t xml:space="preserve">Road: plug-in hybrid cost mixed BEV capital cost with ICEV insurance and maintenance</t>
         </is>
       </c>
       <c r="C246" s="4"/>
@@ -28668,34 +28696,30 @@
       </c>
       <c r="N246" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Withdrawn (not a bug, user 2026-10-29)</t>
+          <t xml:space="preserve">Fixed (v0.9.1 (Coded CPAT) / v0.9.2)</t>
         </is>
       </c>
       <c r="O246" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Withdrawn</t>
+          <t xml:space="preserve">Closed</t>
         </is>
       </c>
       <c r="P246" s="4"/>
-      <c r="Q246" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Mitigation row 4522 (trbusel.bus.ecy), column D</t>
-        </is>
-      </c>
+      <c r="Q246" s="3"/>
       <c r="R246" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Registered in v0.9.1 as a bug (column D = base bus use of diesel, LPG, gas and electricity). Withdrawn by the user (2026-10-29): it is the legacy method (legacy row 5318 sums every bus fuel): bus electricity = all base-year bus energy x the passenger electricity share, which is how buses electrify. The proposed fix (base-year bus electricity only) would keep bus electricity near zero where base-year bus electricity is ~0. Legacy bug L30 (units) stays as it is.</t>
+          <t xml:space="preserve">trtcfp.pas.phv took the BEV depreciation and salvage with the ICEV insurance and maintenance (insurance on the ICEV price).</t>
         </is>
       </c>
       <c r="S246" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">None: kept as legacy.</t>
+          <t xml:space="preserve">One price basis (user 2026-10-29; no PHEV price in the data): new row trimphv.pas.phv, insurance on the BEV price with the ICEV maintenance per km and the ICEV distance. Engineer road model only. In legacy too: L227 (with L41, the range anxiety).</t>
         </is>
       </c>
       <c r="T246" s="3"/>
       <c r="U246" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">L30</t>
+          <t xml:space="preserve">L227, L41</t>
         </is>
       </c>
       <c r="V246" s="3" t="inlineStr">
@@ -28707,12 +28731,12 @@
     <row r="247">
       <c r="A247" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M19</t>
+          <t xml:space="preserve">M18</t>
         </is>
       </c>
       <c r="B247" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nominal GDP divided by a billion although WEO is in billions</t>
+          <t xml:space="preserve">Road: bus electricity scaled by the bus energy of every fuel (withdrawn: not a bug)</t>
         </is>
       </c>
       <c r="C247" s="4"/>
@@ -28752,28 +28776,36 @@
       </c>
       <c r="N247" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fixed (v0.9.1 (Coded CPAT) / v0.9.2)</t>
+          <t xml:space="preserve">Withdrawn (not a bug, user 2026-10-29)</t>
         </is>
       </c>
       <c r="O247" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Closed</t>
+          <t xml:space="preserve">Withdrawn</t>
         </is>
       </c>
       <c r="P247" s="4"/>
-      <c r="Q247" s="3"/>
+      <c r="Q247" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mitigation row 4522 (trbusel.bus.ecy), column D</t>
+        </is>
+      </c>
       <c r="R247" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">gdpn = WEO NGDP / Billion: 1e9 too small (Egypt 7.8e-6 bn LCU). Not in legacy (row 424, no division): introduced in v0.5.6.</t>
+          <t xml:space="preserve">Registered in v0.9.1 as a bug (column D = base bus use of diesel, LPG, gas and electricity). Withdrawn by the user (2026-10-29): it is the legacy method (legacy row 5318 sums every bus fuel): bus electricity = all base-year bus energy x the passenger electricity share, which is how buses electrify. The proposed fix (base-year bus electricity only) would keep bus electricity near zero where base-year bus electricity is ~0. Legacy bug L30 (units) stays as it is.</t>
         </is>
       </c>
       <c r="S247" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">No division; unit bn nominal. Output rows only.</t>
+          <t xml:space="preserve">None: kept as legacy.</t>
         </is>
       </c>
       <c r="T247" s="3"/>
-      <c r="U247" s="3"/>
+      <c r="U247" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L30</t>
+        </is>
+      </c>
       <c r="V247" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Documentation, appendix</t>
@@ -28783,12 +28815,12 @@
     <row r="248">
       <c r="A248" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M20</t>
+          <t xml:space="preserve">M19</t>
         </is>
       </c>
       <c r="B248" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">International prices: World Bank and IEA LNG and Europe gas series swapped</t>
+          <t xml:space="preserve">Nominal GDP divided by a billion although WEO is in billions</t>
         </is>
       </c>
       <c r="C248" s="4"/>
@@ -28840,20 +28872,16 @@
       <c r="Q248" s="3"/>
       <c r="R248" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The WB LNG price read Prices_int row 15 ("Natural gas, Europe") and the Europe price row 17 ("Liquefied natural gas, Japan"); the legacy check found the same swap in the IEA block (rows 39 and 41), which EIA, AVG and IMF-IEA inherit. In legacy too: L228 (WB), L229 (IEA).</t>
+          <t xml:space="preserve">gdpn = WEO NGDP / Billion: 1e9 too small (Egypt 7.8e-6 bn LCU). Not in legacy (row 424, no division): introduced in v0.5.6.</t>
         </is>
       </c>
       <c r="S248" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Each series read by its label: WB LNG row 17, Europe row 15; IEA LNG row 41, Europe row 39. Egypt unchanged (IMF, global gas).</t>
+          <t xml:space="preserve">No division; unit bn nominal. Output rows only.</t>
         </is>
       </c>
       <c r="T248" s="3"/>
-      <c r="U248" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">L228, L229</t>
-        </is>
-      </c>
+      <c r="U248" s="3"/>
       <c r="V248" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Documentation, appendix</t>
@@ -28863,12 +28891,12 @@
     <row r="249">
       <c r="A249" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M21</t>
+          <t xml:space="preserve">M20</t>
         </is>
       </c>
       <c r="B249" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Methane fee: marginal abatement price #DIV/0 where the curve exponent is 0</t>
+          <t xml:space="preserve">International prices: World Bank and IEA LNG and Europe gas series swapped</t>
         </is>
       </c>
       <c r="C249" s="4"/>
@@ -28920,16 +28948,20 @@
       <c r="Q249" s="3"/>
       <c r="R249" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">mfp = MIN(fee, (1/a)^(1/b)) gave #DIV/0 where b = 0 and a &lt;&gt; 0, and #NUM! where b is about 1e-14 (45 country sources in the data, e.g. AFG coal mining; DMA livestock b = 0). Not in legacy (no cap): introduced in v0.3.17.</t>
+          <t xml:space="preserve">The WB LNG price read Prices_int row 15 ("Natural gas, Europe") and the Europe price row 17 ("Liquefied natural gas, Japan"); the legacy check found the same swap in the IEA block (rows 39 and 41), which EIA, AVG and IMF-IEA inherit. In legacy too: L228 (WB), L229 (IEA).</t>
         </is>
       </c>
       <c r="S249" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">IF(a = 0, 0, MIN(fee, IFERROR(a^(-1/b), fee))) (MFEEPRICE): no cap where b = 0 or where the cap overflows (it is beyond any fee there). Egypt unchanged.</t>
+          <t xml:space="preserve">Each series read by its label: WB LNG row 17, Europe row 15; IEA LNG row 41, Europe row 39. Egypt unchanged (IMF, global gas).</t>
         </is>
       </c>
       <c r="T249" s="3"/>
-      <c r="U249" s="3"/>
+      <c r="U249" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L228, L229</t>
+        </is>
+      </c>
       <c r="V249" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Documentation, appendix</t>
@@ -28939,12 +28971,12 @@
     <row r="250">
       <c r="A250" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M22</t>
+          <t xml:space="preserve">M21</t>
         </is>
       </c>
       <c r="B250" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Distribution: percentile recycling rows added a % row to amounts in local currency</t>
+          <t xml:space="preserve">Methane fee: marginal abatement price #DIV/0 where the curve exponent is 0</t>
         </is>
       </c>
       <c r="C250" s="4"/>
@@ -28984,7 +29016,7 @@
       </c>
       <c r="N250" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fixed (v0.9.1 (Coded CPAT) / v0.9.2 (Distribution 0.1.4))</t>
+          <t xml:space="preserve">Fixed (v0.9.1 (Coded CPAT) / v0.9.2)</t>
         </is>
       </c>
       <c r="O250" s="4" t="inlineStr">
@@ -28996,12 +29028,12 @@
       <c r="Q250" s="3"/>
       <c r="R250" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">hrec = (pit + pui + cts + tgt) / hcpc x 100 read the public-investment row by the key pui.&lt;sample&gt;, which the recycling-gain % row reuses, so it added % of consumption to amounts per person.</t>
+          <t xml:space="preserve">mfp = MIN(fee, (1/a)^(1/b)) gave #DIV/0 where b = 0 and a &lt;&gt; 0, and #NUM! where b is about 1e-14 (45 country sources in the data, e.g. AFG coal mining; DMA livestock b = 0). Not in legacy (no cap): introduced in v0.3.17.</t>
         </is>
       </c>
       <c r="S250" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">hrec reads the public investment amount per person of the sample (LCU). Egypt: the 25th/75th percentile recycling and net rows where public investment is used. Not in legacy (T3194 uses the amount): introduced in v0.6.0 (fixes D18, D19).</t>
+          <t xml:space="preserve">IF(a = 0, 0, MIN(fee, IFERROR(a^(-1/b), fee))) (MFEEPRICE): no cap where b = 0 or where the cap overflows (it is beyond any fee there). Egypt unchanged.</t>
         </is>
       </c>
       <c r="T250" s="3"/>
@@ -29015,96 +29047,88 @@
     <row r="251">
       <c r="A251" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DOC1</t>
+          <t xml:space="preserve">M22</t>
         </is>
       </c>
       <c r="B251" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">No in-model GDP feedback equation</t>
+          <t xml:space="preserve">Distribution: percentile recycling rows added a % row to amounts in local currency</t>
         </is>
       </c>
       <c r="C251" s="4"/>
-      <c r="D251" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-10-29</t>
-        </is>
-      </c>
-      <c r="E251" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5 (High)</t>
-        </is>
-      </c>
-      <c r="F251" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No</t>
+      <c r="D251" s="4"/>
+      <c r="E251" s="4"/>
+      <c r="F251" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Solved</t>
         </is>
       </c>
       <c r="G251" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">CPAT-AI (Coded CPAT planning)</t>
-        </is>
-      </c>
-      <c r="H251" s="0"/>
+          <t xml:space="preserve">Stephen (CPAT-AI)</t>
+        </is>
+      </c>
+      <c r="H251" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CPAT-AI (prototype)</t>
+        </is>
+      </c>
       <c r="I251" s="3"/>
       <c r="J251" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Documentation bug</t>
+          <t xml:space="preserve">Prototype bug</t>
         </is>
       </c>
       <c r="K251" s="4"/>
       <c r="L251" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Documentation</t>
+          <t xml:space="preserve">Mitigation</t>
         </is>
       </c>
       <c r="M251" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Documentation</t>
+          <t xml:space="preserve">Mitigation</t>
         </is>
       </c>
       <c r="N251" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not affected</t>
+          <t xml:space="preserve">Fixed (v0.9.1 (Coded CPAT) / v0.9.2 (Distribution 0.1.4))</t>
         </is>
       </c>
       <c r="O251" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open: correct in the methodology documentation (no model change)</t>
+          <t xml:space="preserve">Closed</t>
         </is>
       </c>
       <c r="P251" s="4"/>
-      <c r="Q251" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">04_Multipliers.qmd (whole chapter); 03_Mitigation.qmd Appendix E ("Include endogenous GDP effects?")</t>
-        </is>
-      </c>
+      <c r="Q251" s="3"/>
       <c r="R251" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The multipliers chapter explains how the multipliers are estimated and Appendix E names the option, but no equation shows how the model turns new revenue and its uses into a GDP effect (fiscal space, impulse, multipliers by lag, timing) and feeds it back into energy demand.</t>
+          <t xml:space="preserve">hrec = (pit + pui + cts + tgt) / hcpc x 100 read the public-investment row by the key pui.&lt;sample&gt;, which the recycling-gain % row reuses, so it added % of consumption to amounts per person.</t>
         </is>
       </c>
       <c r="S251" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add the in-model equations: fiscal space, impulse, effect of each use with the multipliers by lag, GDP level one year later (as Excel-AI Equations.md E91-E95).</t>
+          <t xml:space="preserve">hrec reads the public investment amount per person of the sample (LCU). Egypt: the 25th/75th percentile recycling and net rows where public investment is used. Not in legacy (T3194 uses the amount): introduced in v0.6.0 (fixes D18, D19).</t>
         </is>
       </c>
       <c r="T251" s="3"/>
       <c r="U251" s="3"/>
       <c r="V251" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Register; methodology documentation (docs/01_MainDocumentation)</t>
+          <t xml:space="preserve">Documentation, appendix</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DOC2</t>
+          <t xml:space="preserve">DOC1</t>
         </is>
       </c>
       <c r="B252" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Electricity price markup has the wrong sign</t>
+          <t xml:space="preserve">No in-model GDP feedback equation</t>
         </is>
       </c>
       <c r="C252" s="4"/>
@@ -29159,17 +29183,17 @@
       <c r="P252" s="4"/>
       <c r="Q252" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">03_Mitigation.qmd, Power prices &gt; Concept 4: End-user prices, line 1354</t>
+          <t xml:space="preserve">04_Multipliers.qmd (whole chapter); 03_Mitigation.qmd Appendix E ("Include endogenous GDP effects?")</t>
         </is>
       </c>
       <c r="R252" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">mu^T = gnc^av + tmc - hrp is then added to the end-user price p^T; in the base year that gives 2(gnc^av + tmc) - hrp instead of the historical price hrp. The text ("when the markup is negative ... the model captures a subsidy") needs the opposite sign.</t>
+          <t xml:space="preserve">The multipliers chapter explains how the multipliers are estimated and Appendix E names the option, but no equation shows how the model turns new revenue and its uses into a GDP effect (fiscal space, impulse, multipliers by lag, timing) and feeds it back into energy demand.</t>
         </is>
       </c>
       <c r="S252" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">mu^T = hrp - gnc^av - tmc.</t>
+          <t xml:space="preserve">Add the in-model equations: fiscal space, impulse, effect of each use with the multipliers by lag, GDP level one year later (as Excel-AI Equations.md E91-E95).</t>
         </is>
       </c>
       <c r="T252" s="3"/>
@@ -29183,12 +29207,12 @@
     <row r="253">
       <c r="A253" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DOC3</t>
+          <t xml:space="preserve">DOC2</t>
         </is>
       </c>
       <c r="B253" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Discount factor and levelised total investment cost written wrongly</t>
+          <t xml:space="preserve">Electricity price markup has the wrong sign</t>
         </is>
       </c>
       <c r="C253" s="4"/>
@@ -29243,17 +29267,17 @@
       <c r="P253" s="4"/>
       <c r="Q253" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">03_Mitigation.qmd, Power prices &gt; Concept 2: Levelized costs of generation, lines 1253-1255</t>
+          <t xml:space="preserve">03_Mitigation.qmd, Power prices &gt; Concept 4: End-user prices, line 1354</t>
         </is>
       </c>
       <c r="R253" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The discount factor dfc is defined as "1 + wacc^(t - t0)" (should be (1 + wacc)^-(t - t0)), and tic = vc cf dfc / (cf dfc) + fix^fl cancels to vc + fix^fl: the sums over the years are missing.</t>
+          <t xml:space="preserve">mu^T = gnc^av + tmc - hrp is then added to the end-user price p^T; in the base year that gives 2(gnc^av + tmc) - hrp instead of the historical price hrp. The text ("when the markup is negative ... the model captures a subsidy") needs the opposite sign.</t>
         </is>
       </c>
       <c r="S253" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Write dfc = (1 + wacc)^-(t - t0) and tic = sum_t vc_t cf dfc_t / sum_t cf dfc_t + fix^fl.</t>
+          <t xml:space="preserve">mu^T = hrp - gnc^av - tmc.</t>
         </is>
       </c>
       <c r="T253" s="3"/>
@@ -29267,12 +29291,12 @@
     <row r="254">
       <c r="A254" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DOC4</t>
+          <t xml:space="preserve">DOC3</t>
         </is>
       </c>
       <c r="B254" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">GDP elasticity of power demand never defined</t>
+          <t xml:space="preserve">Discount factor and levelised total investment cost written wrongly</t>
         </is>
       </c>
       <c r="C254" s="4"/>
@@ -29283,7 +29307,7 @@
       </c>
       <c r="E254" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 (Medium)</t>
+          <t xml:space="preserve">5 (High)</t>
         </is>
       </c>
       <c r="F254" s="21" t="inlineStr">
@@ -29327,17 +29351,17 @@
       <c r="P254" s="4"/>
       <c r="Q254" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">03_Mitigation.qmd, Engineer model &gt; Power demand (line 1506); Elasticity model &gt; Total power demand (line 1850)</t>
+          <t xml:space="preserve">03_Mitigation.qmd, Power prices &gt; Concept 2: Levelized costs of generation, lines 1253-1255</t>
         </is>
       </c>
       <c r="R254" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Both power-demand equations use epsilon_G, which no notation table defines; the fuel equation uses epsilon_Y.</t>
+          <t xml:space="preserve">The discount factor dfc is defined as "1 + wacc^(t - t0)" (should be (1 + wacc)^-(t - t0)), and tic = vc cf dfc / (cf dfc) + fix^fl cancels to vc + fix^fl: the sums over the years are missing.</t>
         </is>
       </c>
       <c r="S254" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use epsilon_Y (with the income-level adjustment, as the model) or define epsilon_G.</t>
+          <t xml:space="preserve">Write dfc = (1 + wacc)^-(t - t0) and tic = sum_t vc_t cf dfc_t / sum_t cf dfc_t + fix^fl.</t>
         </is>
       </c>
       <c r="T254" s="3"/>
@@ -29351,12 +29375,12 @@
     <row r="255">
       <c r="A255" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DOC5</t>
+          <t xml:space="preserve">DOC4</t>
         </is>
       </c>
       <c r="B255" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Undefined symbol tex in the old power cost model</t>
+          <t xml:space="preserve">GDP elasticity of power demand never defined</t>
         </is>
       </c>
       <c r="C255" s="4"/>
@@ -29367,7 +29391,7 @@
       </c>
       <c r="E255" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 (Low)</t>
+          <t xml:space="preserve">3 (Medium)</t>
         </is>
       </c>
       <c r="F255" s="21" t="inlineStr">
@@ -29411,17 +29435,17 @@
       <c r="P255" s="4"/>
       <c r="Q255" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">03_Mitigation.qmd, Appendix C &gt; Power generation costs, line 4225</t>
+          <t xml:space="preserve">03_Mitigation.qmd, Engineer model &gt; Power demand (line 1506); Elasticity model &gt; Total power demand (line 1850)</t>
         </is>
       </c>
       <c r="R255" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">gnc = efc + nfc + rps + nct (1 - tex): tex is not defined anywhere (presumably a tax-exemption share).</t>
+          <t xml:space="preserve">Both power-demand equations use epsilon_G, which no notation table defines; the fuel equation uses epsilon_Y.</t>
         </is>
       </c>
       <c r="S255" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Define tex or remove the term.</t>
+          <t xml:space="preserve">Use epsilon_Y (with the income-level adjustment, as the model) or define epsilon_G.</t>
         </is>
       </c>
       <c r="T255" s="3"/>
@@ -29435,12 +29459,12 @@
     <row r="256">
       <c r="A256" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DOC6</t>
+          <t xml:space="preserve">DOC5</t>
         </is>
       </c>
       <c r="B256" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Derivative of short-term storage wrong</t>
+          <t xml:space="preserve">Undefined symbol tex in the old power cost model</t>
         </is>
       </c>
       <c r="C256" s="4"/>
@@ -29451,7 +29475,7 @@
       </c>
       <c r="E256" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 (Medium)</t>
+          <t xml:space="preserve">1 (Low)</t>
         </is>
       </c>
       <c r="F256" s="21" t="inlineStr">
@@ -29495,17 +29519,17 @@
       <c r="P256" s="4"/>
       <c r="Q256" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">03_Mitigation.qmd, Storage decision &gt; Short-term storage, line 1730</t>
+          <t xml:space="preserve">03_Mitigation.qmd, Appendix C &gt; Power generation costs, line 4225</t>
         </is>
       </c>
       <c r="R256" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">sst = 9 v^2, but its derivative is written d sst / dv = 18 v^2.</t>
+          <t xml:space="preserve">gnc = efc + nfc + rps + nct (1 - tex): tex is not defined anywhere (presumably a tax-exemption share).</t>
         </is>
       </c>
       <c r="S256" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">d sst / dv = 18 v.</t>
+          <t xml:space="preserve">Define tex or remove the term.</t>
         </is>
       </c>
       <c r="T256" s="3"/>
@@ -29519,12 +29543,12 @@
     <row r="257">
       <c r="A257" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DOC7</t>
+          <t xml:space="preserve">DOC6</t>
         </is>
       </c>
       <c r="B257" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Long-term storage table does not match its formula</t>
+          <t xml:space="preserve">Derivative of short-term storage wrong</t>
         </is>
       </c>
       <c r="C257" s="4"/>
@@ -29579,17 +29603,17 @@
       <c r="P257" s="4"/>
       <c r="Q257" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">03_Mitigation.qmd, Storage decision &gt; Long-term storage, lines 1747-1765</t>
+          <t xml:space="preserve">03_Mitigation.qmd, Storage decision &gt; Short-term storage, line 1730</t>
         </is>
       </c>
       <c r="R257" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">slt = ((v - 0.75)/(1 - 0.75))^2 above 75% VRE, so the marginal requirement is 2(v - 0.75)/0.25^2 (3.2 at 85%); the table gives 2.5 at 85%, 5.0 at 90%, 7.5 at 95%, 10.0 at 100% (a linear rule).</t>
+          <t xml:space="preserve">sst = 9 v^2, but its derivative is written d sst / dv = 18 v^2.</t>
         </is>
       </c>
       <c r="S257" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Make the table and the formula agree (state which one the model uses).</t>
+          <t xml:space="preserve">d sst / dv = 18 v.</t>
         </is>
       </c>
       <c r="T257" s="3"/>
@@ -29603,12 +29627,12 @@
     <row r="258">
       <c r="A258" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DOC8</t>
+          <t xml:space="preserve">DOC7</t>
         </is>
       </c>
       <c r="B258" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Efficiency cost: wrong symbol and wrong description</t>
+          <t xml:space="preserve">Long-term storage table does not match its formula</t>
         </is>
       </c>
       <c r="C258" s="4"/>
@@ -29663,17 +29687,17 @@
       <c r="P258" s="4"/>
       <c r="Q258" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">03_Mitigation.qmd, Efficiency costs in CPAT, lines 2701-2703</t>
+          <t xml:space="preserve">03_Mitigation.qmd, Storage decision &gt; Long-term storage, lines 1747-1765</t>
         </is>
       </c>
       <c r="R258" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The equation uses nc_ft where the text and the rest of the chapter use ncp_ft; the text calls (ncp - xcp)/2 "the average of new and pre-existing tax", but it is half their difference.</t>
+          <t xml:space="preserve">slt = ((v - 0.75)/(1 - 0.75))^2 above 75% VRE, so the marginal requirement is 2(v - 0.75)/0.25^2 (3.2 at 85%); the table gives 2.5 at 85%, 5.0 at 90%, 7.5 at 95%, 10.0 at 100% (a linear rule).</t>
         </is>
       </c>
       <c r="S258" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Write ncp_ft and describe the term as half the difference (the Harberger trapezoid).</t>
+          <t xml:space="preserve">Make the table and the formula agree (state which one the model uses).</t>
         </is>
       </c>
       <c r="T258" s="3"/>
@@ -29687,12 +29711,12 @@
     <row r="259">
       <c r="A259" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DOC9</t>
+          <t xml:space="preserve">DOC8</t>
         </is>
       </c>
       <c r="B259" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Producer subsidies added in one place, subtracted in another</t>
+          <t xml:space="preserve">Efficiency cost: wrong symbol and wrong description</t>
         </is>
       </c>
       <c r="C259" s="4"/>
@@ -29747,17 +29771,17 @@
       <c r="P259" s="4"/>
       <c r="Q259" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">03_Mitigation.qmd, Prices &gt; Overview (line 737) and Appendix C &gt; Calculations (line 4085)</t>
+          <t xml:space="preserve">03_Mitigation.qmd, Efficiency costs in CPAT, lines 2701-2703</t>
         </is>
       </c>
       <c r="R259" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The main text says the supply price is fixed plus floating portions "minus any remaining producer subsidies"; Appendix C writes sp = fixsp + fltsp + ps.</t>
+          <t xml:space="preserve">The equation uses nc_ft where the text and the rest of the chapter use ncp_ft; the text calls (ncp - xcp)/2 "the average of new and pre-existing tax", but it is half their difference.</t>
         </is>
       </c>
       <c r="S259" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">State the sign convention of ps once and use it in both places.</t>
+          <t xml:space="preserve">Write ncp_ft and describe the term as half the difference (the Harberger trapezoid).</t>
         </is>
       </c>
       <c r="T259" s="3"/>
@@ -29771,12 +29795,12 @@
     <row r="260">
       <c r="A260" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DOC10</t>
+          <t xml:space="preserve">DOC9</t>
         </is>
       </c>
       <c r="B260" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Base year and historical price years stated inconsistently</t>
+          <t xml:space="preserve">Producer subsidies added in one place, subtracted in another</t>
         </is>
       </c>
       <c r="C260" s="4"/>
@@ -29787,7 +29811,7 @@
       </c>
       <c r="E260" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 (Low)</t>
+          <t xml:space="preserve">3 (Medium)</t>
         </is>
       </c>
       <c r="F260" s="21" t="inlineStr">
@@ -29831,17 +29855,17 @@
       <c r="P260" s="4"/>
       <c r="Q260" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">03_Mitigation.qmd, Prices &gt; Overview (line 590); Appendix C, lines 4070-4096</t>
+          <t xml:space="preserve">03_Mitigation.qmd, Prices &gt; Overview (line 737) and Appendix C &gt; Calculations (line 4085)</t>
         </is>
       </c>
       <c r="R260" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The overview gives base year 2019 and historical price years 2019-2021; Appendix C averages over 2018-2022, is headed "Forecasted prices (after 2021)" and says "for years starting from 2023".</t>
+          <t xml:space="preserve">The main text says the supply price is fixed plus floating portions "minus any remaining producer subsidies"; Appendix C writes sp = fixsp + fltsp + ps.</t>
         </is>
       </c>
       <c r="S260" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">One statement of the base year and the historical window (the current data vintage), used throughout.</t>
+          <t xml:space="preserve">State the sign convention of ps once and use it in both places.</t>
         </is>
       </c>
       <c r="T260" s="3"/>
@@ -29855,12 +29879,12 @@
     <row r="261">
       <c r="A261" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DOC11</t>
+          <t xml:space="preserve">DOC10</t>
         </is>
       </c>
       <c r="B261" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Capacity stock equation written in generation and summed over fuels</t>
+          <t xml:space="preserve">Base year and historical price years stated inconsistently</t>
         </is>
       </c>
       <c r="C261" s="4"/>
@@ -29871,7 +29895,7 @@
       </c>
       <c r="E261" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 (Medium)</t>
+          <t xml:space="preserve">1 (Low)</t>
         </is>
       </c>
       <c r="F261" s="21" t="inlineStr">
@@ -29915,17 +29939,17 @@
       <c r="P261" s="4"/>
       <c r="Q261" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">03_Mitigation.qmd, Engineer model &gt; Retirement and capacity needed, line 1580</t>
+          <t xml:space="preserve">03_Mitigation.qmd, Prices &gt; Overview (line 590); Appendix C, lines 4070-4096</t>
         </is>
       </c>
       <c r="R261" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">g_ocft = g_ocf,t-1 - sum_f ret_ocf,t-1 + inv: uses generation g (GWh) for capacity and subtracts the retirements of all fuels from a fuel-specific stock; the notation table gives inv and ret in MWh.</t>
+          <t xml:space="preserve">The overview gives base year 2019 and historical price years 2019-2021; Appendix C averages over 2018-2022, is headed "Forecasted prices (after 2021)" and says "for years starting from 2023".</t>
         </is>
       </c>
       <c r="S261" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">cap_ft = cap_f,t-1 - ret_f,t-1 + inv_f,t-1, in MW.</t>
+          <t xml:space="preserve">One statement of the base year and the historical window (the current data vintage), used throughout.</t>
         </is>
       </c>
       <c r="T261" s="3"/>
@@ -29939,12 +29963,12 @@
     <row r="262">
       <c r="A262" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DOC12</t>
+          <t xml:space="preserve">DOC11</t>
         </is>
       </c>
       <c r="B262" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fuel cost of power: text and equation use different prices</t>
+          <t xml:space="preserve">Capacity stock equation written in generation and summed over fuels</t>
         </is>
       </c>
       <c r="C262" s="4"/>
@@ -29999,17 +30023,17 @@
       <c r="P262" s="4"/>
       <c r="Q262" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">03_Mitigation.qmd, Power prices &gt; Concept 1, lines 1197 and 1202</t>
+          <t xml:space="preserve">03_Mitigation.qmd, Engineer model &gt; Retirement and capacity needed, line 1580</t>
         </is>
       </c>
       <c r="R262" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The text says fuel cost = pre-tax price (including producer subsidies) ps / thermal efficiency; the equation writes the retail price p / nu; ps is elsewhere the producer subsidy itself.</t>
+          <t xml:space="preserve">g_ocft = g_ocf,t-1 - sum_f ret_ocf,t-1 + inv: uses generation g (GWh) for capacity and subtracts the retirements of all fuels from a fuel-specific stock; the notation table gives inv and ret in MWh.</t>
         </is>
       </c>
       <c r="S262" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use one symbol for the price that enters (the pre-tax price) in both.</t>
+          <t xml:space="preserve">cap_ft = cap_f,t-1 - ret_f,t-1 + inv_f,t-1, in MW.</t>
         </is>
       </c>
       <c r="T262" s="3"/>
@@ -30023,12 +30047,12 @@
     <row r="263">
       <c r="A263" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DOC13</t>
+          <t xml:space="preserve">DOC12</t>
         </is>
       </c>
       <c r="B263" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Units wrong or inconsistent in the notation tables</t>
+          <t xml:space="preserve">Fuel cost of power: text and equation use different prices</t>
         </is>
       </c>
       <c r="C263" s="4"/>
@@ -30039,7 +30063,7 @@
       </c>
       <c r="E263" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 (Low)</t>
+          <t xml:space="preserve">3 (Medium)</t>
         </is>
       </c>
       <c r="F263" s="21" t="inlineStr">
@@ -30083,17 +30107,17 @@
       <c r="P263" s="4"/>
       <c r="Q263" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">03_Mitigation.qmd, notation tables of Emissions, Fiscal revenues, Engineer model, Power prices</t>
+          <t xml:space="preserve">03_Mitigation.qmd, Power prices &gt; Concept 1, lines 1197 and 1202</t>
         </is>
       </c>
       <c r="R263" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">em in tCO2/GJ (emissions are MtCO2e); ncp in USD/tCO2 in the revenue table but USD/GJ in the price table; lambda_f in GWh (a share); zeta in MWh (text: a percentage); inv, ret in MWh (capacity); dtc and opf per kWh in the table but per kW in the text.</t>
+          <t xml:space="preserve">The text says fuel cost = pre-tax price (including producer subsidies) ps / thermal efficiency; the equation writes the retail price p / nu; ps is elsewhere the producer subsidy itself.</t>
         </is>
       </c>
       <c r="S263" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Correct each unit.</t>
+          <t xml:space="preserve">Use one symbol for the price that enters (the pre-tax price) in both.</t>
         </is>
       </c>
       <c r="T263" s="3"/>
@@ -30107,12 +30131,12 @@
     <row r="264">
       <c r="A264" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DOC14</t>
+          <t xml:space="preserve">DOC13</t>
         </is>
       </c>
       <c r="B264" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Symbol names differ between the text, the tables and the equations</t>
+          <t xml:space="preserve">Units wrong or inconsistent in the notation tables</t>
         </is>
       </c>
       <c r="C264" s="4"/>
@@ -30167,17 +30191,17 @@
       <c r="P264" s="4"/>
       <c r="Q264" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">03_Mitigation.qmd, several sections</t>
+          <t xml:space="preserve">03_Mitigation.qmd, notation tables of Emissions, Fiscal revenues, Engineer model, Power prices</t>
         </is>
       </c>
       <c r="R264" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">opv / vop (variable OpEx); ipc / ip / imp (implicit coal price); revEx / revExi; ct / ctr (price controls); sp_T / sp^T and mu / mu^T; H_f / H_g and K_g; COA / COAL; CF / cf; IPPU Delta em_ocP (text) / Delta em_ocI (equation); LCOE denominator dem / g; rebound term P_t (aggregate price) for p.</t>
+          <t xml:space="preserve">em in tCO2/GJ (emissions are MtCO2e); ncp in USD/tCO2 in the revenue table but USD/GJ in the price table; lambda_f in GWh (a share); zeta in MWh (text: a percentage); inv, ret in MWh (capacity); dtc and opf per kWh in the table but per kW in the text.</t>
         </is>
       </c>
       <c r="S264" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">One name per quantity, as in the notation tables.</t>
+          <t xml:space="preserve">Correct each unit.</t>
         </is>
       </c>
       <c r="T264" s="3"/>
@@ -30191,12 +30215,12 @@
     <row r="265">
       <c r="A265" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DOC15</t>
+          <t xml:space="preserve">DOC14</t>
         </is>
       </c>
       <c r="B265" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Elasticity power model: index roles swapped in the share equation</t>
+          <t xml:space="preserve">Symbol names differ between the text, the tables and the equations</t>
         </is>
       </c>
       <c r="C265" s="4"/>
@@ -30251,17 +30275,17 @@
       <c r="P265" s="4"/>
       <c r="Q265" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">03_Mitigation.qmd, Elasticity model &gt; Total power supply</t>
+          <t xml:space="preserve">03_Mitigation.qmd, several sections</t>
         </is>
       </c>
       <c r="R265" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The documented production-share equation sums over i != f in the numerator and j != f in the denominator; the form described as implemented sums over f != i in both.</t>
+          <t xml:space="preserve">opv / vop (variable OpEx); ipc / ip / imp (implicit coal price); revEx / revExi; ct / ctr (price controls); sp_T / sp^T and mu / mu^T; H_f / H_g and K_g; COA / COAL; CF / cf; IPPU Delta em_ocP (text) / Delta em_ocI (equation); LCOE denominator dem / g; rebound term P_t (aggregate price) for p.</t>
         </is>
       </c>
       <c r="S265" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Write the implemented form once.</t>
+          <t xml:space="preserve">One name per quantity, as in the notation tables.</t>
         </is>
       </c>
       <c r="T265" s="3"/>
@@ -30275,12 +30299,12 @@
     <row r="266">
       <c r="A266" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DOC16</t>
+          <t xml:space="preserve">DOC15</t>
         </is>
       </c>
       <c r="B266" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Distribution: wrong equation reference for direct effects</t>
+          <t xml:space="preserve">Elasticity power model: index roles swapped in the share equation</t>
         </is>
       </c>
       <c r="C266" s="4"/>
@@ -30335,17 +30359,17 @@
       <c r="P266" s="4"/>
       <c r="Q266" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">05_Distribution.qmd, sec 5.3.1, line 384 (eq-5_2, eq-5_3)</t>
+          <t xml:space="preserve">03_Mitigation.qmd, Elasticity model &gt; Total power supply</t>
         </is>
       </c>
       <c r="R266" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Direct effects are said to be "for f=g, in @eq-5_3", but eq-5_3 is the input-output equation with f not in g; the direct effect is the part of eq-5_2 with f in g.</t>
+          <t xml:space="preserve">The documented production-share equation sums over i != f in the numerator and j != f in the denominator; the form described as implemented sums over f != i in both.</t>
         </is>
       </c>
       <c r="S266" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Refer to eq-5_2.</t>
+          <t xml:space="preserve">Write the implemented form once.</t>
         </is>
       </c>
       <c r="T266" s="3"/>
@@ -30359,12 +30383,12 @@
     <row r="267">
       <c r="A267" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DOC17</t>
+          <t xml:space="preserve">DOC16</t>
         </is>
       </c>
       <c r="B267" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fuel codes: electricity coded two ways, biofuel labels swapped</t>
+          <t xml:space="preserve">Distribution: wrong equation reference for direct effects</t>
         </is>
       </c>
       <c r="C267" s="4"/>
@@ -30419,17 +30443,17 @@
       <c r="P267" s="4"/>
       <c r="Q267" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">03_Mitigation.qmd Appendix F (lines 3725-3727, 4765-4767); 05_Distribution.qmd tbl-5_1</t>
+          <t xml:space="preserve">05_Distribution.qmd, sec 5.3.1, line 384 (eq-5_2, eq-5_3)</t>
         </is>
       </c>
       <c r="R267" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Electricity is ecy in the mitigation codes and ely in distribution; Appendix F labels bgs "biodiesel" and bdi "biogasoline", the reverse of the model (bgs biogasoline, bdi biodiesel).</t>
+          <t xml:space="preserve">Direct effects are said to be "for f=g, in @eq-5_3", but eq-5_3 is the input-output equation with f not in g; the direct effect is the part of eq-5_2 with f in g.</t>
         </is>
       </c>
       <c r="S267" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ecy everywhere; bgs biogasoline, bdi biodiesel (also in the codes map).</t>
+          <t xml:space="preserve">Refer to eq-5_2.</t>
         </is>
       </c>
       <c r="T267" s="3"/>
@@ -30443,12 +30467,12 @@
     <row r="268">
       <c r="A268" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DOC18</t>
+          <t xml:space="preserve">DOC17</t>
         </is>
       </c>
       <c r="B268" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Air pollution: index definitions inconsistent</t>
+          <t xml:space="preserve">Fuel codes: electricity coded two ways, biofuel labels swapped</t>
         </is>
       </c>
       <c r="C268" s="4"/>
@@ -30503,17 +30527,17 @@
       <c r="P268" s="4"/>
       <c r="Q268" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">06_Air_pollution.qmd, eq-deltae, eq-ifeach, eq-pomincfactor</t>
+          <t xml:space="preserve">03_Mitigation.qmd Appendix F (lines 3725-3727, 4765-4767); 05_Distribution.qmd tbl-5_1</t>
         </is>
       </c>
       <c r="R268" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">eq-deltae defines k as "pollutant" but uses it to index source regions; eq-ifeach writes iF_{p,j,l} on the left and iF_{p,j,c} in the definitions; eq-pomincfactor mixes d_{POM,2} and delta_{POM,1}.</t>
+          <t xml:space="preserve">Electricity is ecy in the mitigation codes and ely in distribution; Appendix F labels bgs "biodiesel" and bdi "biogasoline", the reverse of the model (bgs biogasoline, bdi biodiesel).</t>
         </is>
       </c>
       <c r="S268" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Correct the index definitions.</t>
+          <t xml:space="preserve">ecy everywhere; bgs biogasoline, bdi biodiesel (also in the codes map).</t>
         </is>
       </c>
       <c r="T268" s="3"/>
@@ -30527,12 +30551,12 @@
     <row r="269">
       <c r="A269" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DOC19</t>
+          <t xml:space="preserve">DOC18</t>
         </is>
       </c>
       <c r="B269" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Road transport: base forecast equation dimensionally ambiguous</t>
+          <t xml:space="preserve">Air pollution: index definitions inconsistent</t>
         </is>
       </c>
       <c r="C269" s="4"/>
@@ -30587,17 +30611,17 @@
       <c r="P269" s="4"/>
       <c r="Q269" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">07_Road_Transport.qmd, eq-basefor</t>
+          <t xml:space="preserve">06_Air_pollution.qmd, eq-deltae, eq-ifeach, eq-pomincfactor</t>
         </is>
       </c>
       <c r="R269" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The base forecast subtracts the average growth rate from a gross growth ratio GDP_t/GDP_t-1, so the result reads as about 1 - g + g_t rather than 1 + g_t - g.</t>
+          <t xml:space="preserve">eq-deltae defines k as "pollutant" but uses it to index source regions; eq-ifeach writes iF_{p,j,l} on the left and iF_{p,j,c} in the definitions; eq-pomincfactor mixes d_{POM,2} and delta_{POM,1}.</t>
         </is>
       </c>
       <c r="S269" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Write the growth terms on one basis.</t>
+          <t xml:space="preserve">Correct the index definitions.</t>
         </is>
       </c>
       <c r="T269" s="3"/>
@@ -30611,12 +30635,12 @@
     <row r="270">
       <c r="A270" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DOC20</t>
+          <t xml:space="preserve">DOC19</t>
         </is>
       </c>
       <c r="B270" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Letters with several meanings</t>
+          <t xml:space="preserve">Road transport: base forecast equation dimensionally ambiguous</t>
         </is>
       </c>
       <c r="C270" s="4"/>
@@ -30671,17 +30695,17 @@
       <c r="P270" s="4"/>
       <c r="Q270" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">All chapters (list: notation_from_methodology.md section 4.1)</t>
+          <t xml:space="preserve">07_Road_Transport.qmd, eq-basefor</t>
         </is>
       </c>
       <c r="R270" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">g is the sector group, generation, a growth rate, the consumption category and a PIT gain; gamma has six meanings; E is electricity, power demand and the energy UNFCCC sector; p/P, j and i also change meaning. Readers cannot tell which is meant without the context.</t>
+          <t xml:space="preserve">The base forecast subtracts the average growth rate from a gross growth ratio GDP_t/GDP_t-1, so the result reads as about 1 - g + g_t rather than 1 + g_t - g.</t>
         </is>
       </c>
       <c r="S270" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">One meaning per letter within a chapter; a notation table per chapter.</t>
+          <t xml:space="preserve">Write the growth terms on one basis.</t>
         </is>
       </c>
       <c r="T270" s="3"/>
@@ -30692,8 +30716,92 @@
         </is>
       </c>
     </row>
+    <row r="271">
+      <c r="A271" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DOC20</t>
+        </is>
+      </c>
+      <c r="B271" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Letters with several meanings</t>
+        </is>
+      </c>
+      <c r="C271" s="4"/>
+      <c r="D271" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-29</t>
+        </is>
+      </c>
+      <c r="E271" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 (Low)</t>
+        </is>
+      </c>
+      <c r="F271" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="G271" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CPAT-AI (Coded CPAT planning)</t>
+        </is>
+      </c>
+      <c r="H271" s="0"/>
+      <c r="I271" s="3"/>
+      <c r="J271" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documentation bug</t>
+        </is>
+      </c>
+      <c r="K271" s="4"/>
+      <c r="L271" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documentation</t>
+        </is>
+      </c>
+      <c r="M271" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documentation</t>
+        </is>
+      </c>
+      <c r="N271" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not affected</t>
+        </is>
+      </c>
+      <c r="O271" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open: correct in the methodology documentation (no model change)</t>
+        </is>
+      </c>
+      <c r="P271" s="4"/>
+      <c r="Q271" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">All chapters (list: notation_from_methodology.md section 4.1)</t>
+        </is>
+      </c>
+      <c r="R271" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">g is the sector group, generation, a growth rate, the consumption category and a PIT gain; gamma has six meanings; E is electricity, power demand and the energy UNFCCC sector; p/P, j and i also change meaning. Readers cannot tell which is meant without the context.</t>
+        </is>
+      </c>
+      <c r="S271" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">One meaning per letter within a chapter; a notation table per chapter.</t>
+        </is>
+      </c>
+      <c r="T271" s="3"/>
+      <c r="U271" s="3"/>
+      <c r="V271" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Register; methodology documentation (docs/01_MainDocumentation)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:V270"/>
+  <autoFilter ref="A1:V271"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>